<commit_message>
Atualiza modelo de planilha com coluna centro de custo
</commit_message>
<xml_diff>
--- a/public/modelo-importacao-veiculos.xlsx
+++ b/public/modelo-importacao-veiculos.xlsx
@@ -200,6 +200,11 @@
         <t>Opcional. Nome completo de um condutor ja cadastrado em /usuarios. Se nao encontrar, o veiculo e criado sem condutor.</t>
       </text>
     </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Codigo ou nome do centro de custo do veiculo (texto livre).</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -493,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -503,6 +508,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,6 +547,11 @@
           <t>Condutor</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Centro de custo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -572,6 +583,11 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Joao da Silva</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1234</t>
         </is>
       </c>
     </row>

</xml_diff>